<commit_message>
Redesigned time pill and fixed a few things in p7
</commit_message>
<xml_diff>
--- a/resources/practica6/tiempos.xlsx
+++ b/resources/practica6/tiempos.xlsx
@@ -1,20 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\informatica-30717.github.io\resources\practica6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DB97AD1-460C-4ACA-BE44-A37DEFF88EFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33F9F1DE-1FA8-402D-9C83-1D2825EA0FD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B7D39335-D069-4A90-893C-03F30C90014F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B7D39335-D069-4A90-893C-03F30C90014F}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlchart.v1.0" hidden="1">Hoja1!$A$2:$A$5</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">Hoja1!$B$1</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">Hoja1!$B$2:$B$5</definedName>
+    <definedName name="_xlchart.v1.3" hidden="1">Hoja1!$C$1</definedName>
+    <definedName name="_xlchart.v1.4" hidden="1">Hoja1!$C$2:$C$5</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -27,9 +34,10 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -48,7 +56,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -178,7 +186,7 @@
         </c:manualLayout>
       </c:layout>
       <c:lineChart>
-        <c:grouping val="stacked"/>
+        <c:grouping val="standard"/>
         <c:varyColors val="0"/>
         <c:ser>
           <c:idx val="0"/>
@@ -1575,13 +1583,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9A9A09A-5E28-40E8-BDEC-E7C7E5B0B536}">
   <dimension ref="A1:H9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="16.44140625" customWidth="1"/>
+    <col min="1" max="1" width="12.625" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="16.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="15">
       <c r="A1" s="6"/>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -1592,7 +1600,7 @@
       <c r="D1" s="5"/>
       <c r="E1" s="5"/>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="15">
       <c r="A2" s="4">
         <v>100</v>
       </c>
@@ -1603,7 +1611,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="15">
       <c r="A3" s="4">
         <v>1000</v>
       </c>
@@ -1614,7 +1622,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="15">
       <c r="A4" s="4">
         <v>10000</v>
       </c>
@@ -1625,7 +1633,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="15">
       <c r="A5" s="4">
         <v>100000</v>
       </c>
@@ -1637,7 +1645,7 @@
       </c>
       <c r="H5" s="3"/>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8">
       <c r="B9" s="3"/>
     </row>
   </sheetData>

</xml_diff>